<commit_message>
update to show apps and directionality of data
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scdoe-my.sharepoint.com/personal/wcothran_ed_sc_gov/Documents/Delete/Claude_Code/gps-ecosystem-visual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{E97CDB31-AE9D-4C9A-89D9-7D4DBC6C9518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93E7D1D1-A38B-4A5C-A7CC-CE8759F84665}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AB047A7-BA9B-43C9-823B-84259A934931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6126C415-B466-49E1-AF6D-20CC7A56C3B7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E83F3718-D06B-4A39-B1A3-1B081857B74B}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="126">
   <si>
     <t>Section</t>
   </si>
@@ -57,6 +57,12 @@
     <t>Future</t>
   </si>
   <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Flow</t>
+  </si>
+  <si>
     <t>Dashboards</t>
   </si>
   <si>
@@ -111,6 +117,12 @@
     <t>Student-level decision-support app for classroom teachers. Student, Classroom, Grade Level, and Section disaggregations of student performance dashboards. Expected growth projections for students; grouping feature for interventions.</t>
   </si>
   <si>
+    <t>App</t>
+  </si>
+  <si>
+    <t>Out</t>
+  </si>
+  <si>
     <t>Student View; Class View; Grade View; Group View</t>
   </si>
   <si>
@@ -120,6 +132,9 @@
     <t>School and district leader app with aggregate data and drill-down dashboards. Allows for analysis of enrollment, attendance, behavior, assessments, grades, and accountability indicators.</t>
   </si>
   <si>
+    <t>Profile; Chronic Absenteeism; Enrollment; Behavior; Assessment; Course Grades; On-Track &amp; CCR; Predictions</t>
+  </si>
+  <si>
     <t>https://scdoe.sharepoint.com/:w:/s/X-TeamGPSGrowingPathwaysforStudents_Group/IQBu-joU23DHT4uYeTMIV_9_AbUuGDtnaZ08lrJPb-vsaM0?e=OoI1nh</t>
   </si>
   <si>
@@ -141,6 +156,9 @@
     <t>App portal for SCDE and LEA users. Content spans HR functions and Grant Reporting to Data Reports and Support Requests.</t>
   </si>
   <si>
+    <t>Bidirectional</t>
+  </si>
+  <si>
     <t>Outputs</t>
   </si>
   <si>
@@ -150,6 +168,9 @@
     <t>School accountability reports published annually.</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
     <t>Funding Data</t>
   </si>
   <si>
@@ -174,6 +195,9 @@
     <t>A planned app-store model: vetted SCDE offices or partners publish data services on the GPS platform.</t>
   </si>
   <si>
+    <t>Service</t>
+  </si>
+  <si>
     <t>State Navigator</t>
   </si>
   <si>
@@ -189,6 +213,9 @@
     <t>Single sign-on and rostering provider. Pushes identity/roster data into connected apps.</t>
   </si>
   <si>
+    <t>In</t>
+  </si>
+  <si>
     <t>Palmetto Pathways</t>
   </si>
   <si>
@@ -391,25 +418,13 @@
   </si>
   <si>
     <t>Who keeps the ecosystem coherent across SCDE divisions and partners.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Student Profile; Chronic Absenteeism; Enrollment; Behavior; Assessment; Course Grades; On-Track &amp; CCR; PreAccountability; On-Track; College &amp; Career Readiness; Attendance; Growth &amp; Predicted Growth; Accountability Metric Comparisons; Accountability Predictions &amp; Targets; Section Profile </t>
-  </si>
-  <si>
-    <t>https://scdoe-my.sharepoint.com/:w:/g/personal/wcothran_ed_sc_gov/IQAYdYDIfSNQRI6fulwpubhrAbyaDQdZxxi5IcBr8VT4w4o?e=E67sD2</t>
-  </si>
-  <si>
-    <t>https://scdoe-my.sharepoint.com/:w:/g/personal/wcothran_ed_sc_gov/IQCcQvWVpilrTb9XiSWkyQ4CARS8Epi8Q0izkbvPHObgxok?e=A17I8k</t>
-  </si>
-  <si>
-    <t>https://scdoe-my.sharepoint.com/:w:/g/personal/wcothran_ed_sc_gov/IQDkec1PjIOfTaHqNW5FOzU1AfhZyvYGgjaHHshW6glfMLk?e=CDb6Fz</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -421,14 +436,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -457,11 +464,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -476,10 +482,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -811,21 +815,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E518B1-1318-4B6E-B6C8-CF66F4009913}">
-  <dimension ref="A1:H37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3CE46A7-A3C6-4CC9-BC6F-D98B3DA40526}">
+  <dimension ref="A1:J37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.6328125" customWidth="1"/>
     <col min="2" max="2" width="28.6328125" customWidth="1"/>
     <col min="3" max="3" width="18.6328125" customWidth="1"/>
-    <col min="4" max="4" width="80.6328125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="10.6328125" customWidth="1"/>
-    <col min="6" max="6" width="40.6328125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="50.6328125" customWidth="1"/>
-    <col min="8" max="8" width="8.6328125" customWidth="1"/>
+    <col min="4" max="4" width="70.6328125" style="4" customWidth="1"/>
+    <col min="5" max="6" width="9.6328125" customWidth="1"/>
+    <col min="7" max="7" width="14.6328125" customWidth="1"/>
+    <col min="8" max="8" width="40.6328125" style="4" customWidth="1"/>
+    <col min="9" max="9" width="50.6328125" customWidth="1"/>
+    <col min="10" max="10" width="8.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -841,692 +846,845 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H2">
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="b">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="4" t="s">
+    <row r="7" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>22</v>
       </c>
-      <c r="E6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>20</v>
-      </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
         <v>25</v>
-      </c>
-      <c r="E7" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>117</v>
       </c>
       <c r="G7" t="s">
         <v>26</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="H8">
+      <c r="F8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" t="s">
+        <v>26</v>
+      </c>
+      <c r="J8">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
-      <c r="H9">
+      <c r="F9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" t="s">
+        <v>38</v>
+      </c>
+      <c r="J9">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
       </c>
-      <c r="H10">
+      <c r="F10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
       </c>
-      <c r="H11">
+      <c r="F11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D12" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" t="s">
+        <v>26</v>
+      </c>
+      <c r="J12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>39</v>
       </c>
-      <c r="E12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>33</v>
-      </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
       </c>
-      <c r="H13">
+      <c r="F13" t="s">
+        <v>42</v>
+      </c>
+      <c r="G13" t="s">
+        <v>26</v>
+      </c>
+      <c r="J13">
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
       </c>
-      <c r="H14">
+      <c r="F14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" t="s">
+        <v>38</v>
+      </c>
+      <c r="J14">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
       </c>
-      <c r="H15">
+      <c r="F15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" t="s">
+        <v>26</v>
+      </c>
+      <c r="J15">
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
       </c>
-      <c r="H16">
+      <c r="F16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" t="s">
+        <v>57</v>
+      </c>
+      <c r="J16">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="D17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" t="s">
+        <v>38</v>
+      </c>
+      <c r="J17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" t="s">
         <v>51</v>
       </c>
-      <c r="E17" t="b">
-        <v>0</v>
-      </c>
-      <c r="H17">
+      <c r="G18" t="s">
+        <v>57</v>
+      </c>
+      <c r="J18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" t="s">
+        <v>38</v>
+      </c>
+      <c r="J19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" t="s">
+        <v>38</v>
+      </c>
+      <c r="J20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" t="s">
+        <v>51</v>
+      </c>
+      <c r="G21" t="s">
+        <v>38</v>
+      </c>
+      <c r="J21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>69</v>
+      </c>
+      <c r="B22" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E22" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" t="s">
+        <v>42</v>
+      </c>
+      <c r="G22" t="s">
+        <v>57</v>
+      </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" t="s">
+        <v>72</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E23" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s">
+        <v>42</v>
+      </c>
+      <c r="G23" t="s">
+        <v>57</v>
+      </c>
+      <c r="J23">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>46</v>
-      </c>
-      <c r="B18" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E18" t="b">
-        <v>0</v>
-      </c>
-      <c r="H18">
+    <row r="24" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>69</v>
+      </c>
+      <c r="B24" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" t="s">
+        <v>42</v>
+      </c>
+      <c r="G24" t="s">
+        <v>57</v>
+      </c>
+      <c r="J24">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>46</v>
-      </c>
-      <c r="B19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" t="b">
-        <v>0</v>
-      </c>
-      <c r="H19">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" t="s">
+        <v>42</v>
+      </c>
+      <c r="G25" t="s">
+        <v>57</v>
+      </c>
+      <c r="J25">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" s="4" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" t="s">
+        <v>78</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E26" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" t="s">
+        <v>42</v>
+      </c>
+      <c r="G26" t="s">
         <v>57</v>
       </c>
-      <c r="E20" t="b">
-        <v>0</v>
-      </c>
-      <c r="H20">
+      <c r="J26">
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E21" t="b">
-        <v>0</v>
-      </c>
-      <c r="H21">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" t="s">
+        <v>42</v>
+      </c>
+      <c r="G27" t="s">
+        <v>57</v>
+      </c>
+      <c r="J27">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>60</v>
-      </c>
-      <c r="B22" t="s">
-        <v>61</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E22" t="b">
-        <v>0</v>
-      </c>
-      <c r="H22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B23" t="s">
-        <v>63</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" t="b">
-        <v>0</v>
-      </c>
-      <c r="H23">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>60</v>
-      </c>
-      <c r="B24" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E24" t="b">
-        <v>0</v>
-      </c>
-      <c r="H24">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>60</v>
-      </c>
-      <c r="B25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E25" t="b">
-        <v>0</v>
-      </c>
-      <c r="H25">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" t="s">
+    <row r="28" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>69</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E26" t="b">
-        <v>0</v>
-      </c>
-      <c r="H26">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>60</v>
-      </c>
-      <c r="B27" t="s">
-        <v>71</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E27" t="b">
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>60</v>
-      </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
       </c>
-      <c r="H28">
+      <c r="F28" t="s">
+        <v>42</v>
+      </c>
+      <c r="G28" t="s">
+        <v>57</v>
+      </c>
+      <c r="J28">
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
       </c>
-      <c r="H29">
+      <c r="F29" t="s">
+        <v>42</v>
+      </c>
+      <c r="G29" t="s">
+        <v>57</v>
+      </c>
+      <c r="J29">
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B30" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="E30" t="b">
         <v>1</v>
       </c>
-      <c r="H30">
+      <c r="F30" t="s">
+        <v>42</v>
+      </c>
+      <c r="G30" t="s">
+        <v>57</v>
+      </c>
+      <c r="J30">
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="B31" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="C31" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
       </c>
-      <c r="G31" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="H31">
+      <c r="J31">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="B32" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="C32" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
       </c>
-      <c r="H32">
+      <c r="J32">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="B33" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="C33" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="D33" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E33" t="b">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>88</v>
       </c>
-      <c r="E33" t="b">
-        <v>0</v>
-      </c>
-      <c r="H33">
+      <c r="B34" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" t="s">
+        <v>99</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E34" t="b">
+        <v>0</v>
+      </c>
+      <c r="J34">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>101</v>
+      </c>
+      <c r="B35" t="s">
+        <v>102</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E35" t="b">
+        <v>0</v>
+      </c>
+      <c r="J35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" t="s">
+        <v>104</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E36" t="b">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>101</v>
+      </c>
+      <c r="B37" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E37" t="b">
+        <v>0</v>
+      </c>
+      <c r="J37">
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>79</v>
-      </c>
-      <c r="B34" t="s">
-        <v>89</v>
-      </c>
-      <c r="C34" t="s">
-        <v>90</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="E34" t="b">
-        <v>0</v>
-      </c>
-      <c r="H34">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>92</v>
-      </c>
-      <c r="B35" t="s">
-        <v>93</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E35" t="b">
-        <v>0</v>
-      </c>
-      <c r="H35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>92</v>
-      </c>
-      <c r="B36" t="s">
-        <v>95</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="E36" t="b">
-        <v>0</v>
-      </c>
-      <c r="H36">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>92</v>
-      </c>
-      <c r="B37" t="s">
-        <v>97</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="E37" t="b">
-        <v>0</v>
-      </c>
-      <c r="H37">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid section" error="Pick one of: Audiences,Tools &amp; Apps,Data Services,Foundation,Governance,Outputs,Inputs" sqref="A2:A500" xr:uid="{4FE4773C-04C0-419F-BE92-3152DC736A77}">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid section" error="Pick one of: Audiences,Tools &amp; Apps,Data Services,Foundation,Governance,Outputs,Inputs" sqref="A2:A500" xr:uid="{08F9F83A-EBAE-46F6-BF44-17D5B9C6E40E}">
       <formula1>"Audiences,Tools &amp; Apps,Data Services,Foundation,Governance,Outputs,Inputs"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E500" xr:uid="{4B227FD9-4EEB-47DB-B65F-E75A6AD2F22E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E500" xr:uid="{C472B2EF-8B33-42E0-BFBA-B14AF61FD5D6}">
       <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid type" error="Pick one of: App,Data,Service (or leave blank)" sqref="F2:F500" xr:uid="{C232765D-62CB-4E31-AB80-447C44417EC4}">
+      <formula1>"App,Data,Service"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid flow" error="Pick one of: In,Out,Bidirectional (or leave blank)" sqref="G2:G500" xr:uid="{C5082321-CB09-41DC-B47F-1AADB255D1E2}">
+      <formula1>"In,Out,Bidirectional"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1534,7 +1692,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ABF28DE-9E70-4103-BBBC-4DBF035B4AAC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D2EFF6-3A8C-4205-945A-5F0E78C87367}">
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1544,83 +1702,77 @@
   <sheetData>
     <row r="1" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{2704e2c5-29f5-4f7e-b91c-bd56f0685995}" enabled="0" method="" siteId="{2704e2c5-29f5-4f7e-b91c-bd56f0685995}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>